<commit_message>
rs2(walls): the K0 each file declares follows its tag again
`apply_tag_k0` writes a corpus file's main!D16 from the test tag that names it, so
a row's file states the K0 its lock was cut at and nothing else. Re-locking the
family moved four tags and dropped one, and the eight workbooks were still
carrying the old pattern: RS2-54's file had no K0 for a tag that now asks for one,
and RS2-52's declared one no tag asks for any more. Rebuilt, so the four locked
rows declare K0 = 1 and the four reported ones declare none.

--roundtrip: 75 passed, 0 failed, 1 error — rs2.md's certified hash, which is the
coordinator's to refresh. verify_rebuild 297/301, the same four that already
differed on fa810bfc.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/verification/files/rocscience/vp087_fem.xlsx
+++ b/docs/verification/files/rocscience/vp087_fem.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/.claude/worktrees/joints-r1/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42723C2E-F56A-D348-AC02-78080B1F6523}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9855A05C-E080-7E4F-9B02-CD939BBA37C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9960" yWindow="2320" windowWidth="30380" windowHeight="22500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4280" yWindow="2000" windowWidth="40460" windowHeight="22500" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="329">
   <si>
     <t>XSLOPE Input Template</t>
   </si>
@@ -1159,6 +1159,15 @@
   </si>
   <si>
     <t>Slip joints (interfaces with no reinforcement)</t>
+  </si>
+  <si>
+    <t>c_res</t>
+  </si>
+  <si>
+    <t>phi_res</t>
+  </si>
+  <si>
+    <t>dil</t>
   </si>
 </sst>
 </file>
@@ -1666,7 +1675,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="38">
+  <dxfs count="37">
     <dxf>
       <fill>
         <patternFill>
@@ -1699,13 +1708,6 @@
       <fill>
         <patternFill>
           <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2227,16 +2229,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>308428</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>172358</xdr:rowOff>
+      <xdr:rowOff>172357</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
+      <xdr:col>20</xdr:col>
       <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>81643</xdr:rowOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>172356</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -2251,8 +2253,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9760857" y="571501"/>
-          <a:ext cx="3701143" cy="1505856"/>
+          <a:off x="12237357" y="571500"/>
+          <a:ext cx="3701143" cy="1995713"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2334,6 +2336,23 @@
           </a:r>
         </a:p>
         <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
             <a:t>phi</a:t>
@@ -2344,13 +2363,94 @@
           </a:r>
         </a:p>
         <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>c_res</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = residual joint cohesion (blank = same as c)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>phi_res</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = residual joint friction angle (blank = same as phi)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>dil</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = joint dilation angle, degrees (blank = 0)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
             <a:t>t_cut</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
-            <a:t> = tension cutoff</a:t>
+            <a:t> = tension cutoff (blank = 0)</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -5445,15 +5545,15 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C676759-96FB-7F49-B49A-BD8077ECE53B}">
-  <dimension ref="A2:O32"/>
+  <dimension ref="A2:R52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.83203125" style="1" customWidth="1"/>
-    <col min="2" max="12" width="10.83203125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="4.33203125" customWidth="1"/>
+    <col min="2" max="15" width="10.83203125" style="1" customWidth="1"/>
+    <col min="16" max="16" width="4.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>193</v>
       </c>
@@ -5479,23 +5579,32 @@
         <v>323</v>
       </c>
       <c r="I2" s="28" t="s">
+        <v>326</v>
+      </c>
+      <c r="J2" s="28" t="s">
+        <v>327</v>
+      </c>
+      <c r="K2" s="28" t="s">
+        <v>328</v>
+      </c>
+      <c r="L2" s="28" t="s">
         <v>120</v>
       </c>
-      <c r="J2" s="28" t="s">
+      <c r="M2" s="28" t="s">
         <v>320</v>
       </c>
-      <c r="K2" s="28" t="s">
+      <c r="N2" s="28" t="s">
         <v>321</v>
       </c>
-      <c r="L2" s="28" t="s">
+      <c r="O2" s="28" t="s">
         <v>322</v>
       </c>
-      <c r="N2" s="29"/>
-      <c r="O2" s="9" t="s">
+      <c r="Q2" s="29"/>
+      <c r="R2" s="9" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -5521,15 +5630,18 @@
         <v>34.0</v>
       </c>
       <c r="I3" s="3"/>
-      <c r="J3" s="3">
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3">
         <v>100000.0</v>
       </c>
-      <c r="K3" s="3">
+      <c r="N3" s="3">
         <v>100000.0</v>
       </c>
-      <c r="L3" s="3"/>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O3" s="3"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -5555,15 +5667,18 @@
         <v>34.0</v>
       </c>
       <c r="I4" s="3"/>
-      <c r="J4" s="3">
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3">
         <v>100000.0</v>
       </c>
-      <c r="K4" s="3">
+      <c r="N4" s="3">
         <v>100000.0</v>
       </c>
-      <c r="L4" s="3"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O4" s="3"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -5589,15 +5704,18 @@
         <v>34.0</v>
       </c>
       <c r="I5" s="3"/>
-      <c r="J5" s="3">
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3">
         <v>100000.0</v>
       </c>
-      <c r="K5" s="3">
+      <c r="N5" s="3">
         <v>100000.0</v>
       </c>
-      <c r="L5" s="3"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O5" s="3"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -5623,15 +5741,18 @@
         <v>34.0</v>
       </c>
       <c r="I6" s="3"/>
-      <c r="J6" s="3">
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3">
         <v>100000.0</v>
       </c>
-      <c r="K6" s="3">
+      <c r="N6" s="3">
         <v>100000.0</v>
       </c>
-      <c r="L6" s="3"/>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O6" s="3"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -5657,15 +5778,18 @@
         <v>34.0</v>
       </c>
       <c r="I7" s="3"/>
-      <c r="J7" s="3">
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3">
         <v>100000.0</v>
       </c>
-      <c r="K7" s="3">
+      <c r="N7" s="3">
         <v>100000.0</v>
       </c>
-      <c r="L7" s="3"/>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O7" s="3"/>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -5691,15 +5815,18 @@
         <v>34.0</v>
       </c>
       <c r="I8" s="3"/>
-      <c r="J8" s="3">
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3">
         <v>100000.0</v>
       </c>
-      <c r="K8" s="3">
+      <c r="N8" s="3">
         <v>100000.0</v>
       </c>
-      <c r="L8" s="3"/>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O8" s="3"/>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -5725,15 +5852,18 @@
         <v>34.0</v>
       </c>
       <c r="I9" s="3"/>
-      <c r="J9" s="3">
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="3">
         <v>100000.0</v>
       </c>
-      <c r="K9" s="3">
+      <c r="N9" s="3">
         <v>100000.0</v>
       </c>
-      <c r="L9" s="3"/>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O9" s="3"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -5759,15 +5889,18 @@
         <v>34.0</v>
       </c>
       <c r="I10" s="3"/>
-      <c r="J10" s="3">
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="M10" s="3">
         <v>100000.0</v>
       </c>
-      <c r="K10" s="3">
+      <c r="N10" s="3">
         <v>100000.0</v>
       </c>
-      <c r="L10" s="3"/>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O10" s="3"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -5793,15 +5926,18 @@
         <v>34.0</v>
       </c>
       <c r="I11" s="3"/>
-      <c r="J11" s="3">
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="3"/>
+      <c r="M11" s="3">
         <v>100000.0</v>
       </c>
-      <c r="K11" s="3">
+      <c r="N11" s="3">
         <v>100000.0</v>
       </c>
-      <c r="L11" s="3"/>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O11" s="3"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>10</v>
       </c>
@@ -5827,15 +5963,18 @@
         <v>34.0</v>
       </c>
       <c r="I12" s="3"/>
-      <c r="J12" s="3">
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+      <c r="L12" s="3"/>
+      <c r="M12" s="3">
         <v>100000.0</v>
       </c>
-      <c r="K12" s="3">
+      <c r="N12" s="3">
         <v>100000.0</v>
       </c>
-      <c r="L12" s="3"/>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O12" s="3"/>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>11</v>
       </c>
@@ -5861,15 +6000,18 @@
         <v>34.0</v>
       </c>
       <c r="I13" s="3"/>
-      <c r="J13" s="3">
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="3"/>
+      <c r="M13" s="3">
         <v>100000.0</v>
       </c>
-      <c r="K13" s="3">
+      <c r="N13" s="3">
         <v>100000.0</v>
       </c>
-      <c r="L13" s="3"/>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O13" s="3"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>12</v>
       </c>
@@ -5895,15 +6037,18 @@
         <v>34.0</v>
       </c>
       <c r="I14" s="3"/>
-      <c r="J14" s="3">
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
+      <c r="M14" s="3">
         <v>100000.0</v>
       </c>
-      <c r="K14" s="3">
+      <c r="N14" s="3">
         <v>100000.0</v>
       </c>
-      <c r="L14" s="3"/>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O14" s="3"/>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>13</v>
       </c>
@@ -5929,15 +6074,18 @@
         <v>34.0</v>
       </c>
       <c r="I15" s="3"/>
-      <c r="J15" s="3">
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="3"/>
+      <c r="M15" s="3">
         <v>100000.0</v>
       </c>
-      <c r="K15" s="3">
+      <c r="N15" s="3">
         <v>100000.0</v>
       </c>
-      <c r="L15" s="3"/>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="O15" s="3"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>14</v>
       </c>
@@ -5963,15 +6111,18 @@
         <v>34.0</v>
       </c>
       <c r="I16" s="3"/>
-      <c r="J16" s="3">
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+      <c r="L16" s="3"/>
+      <c r="M16" s="3">
         <v>100000.0</v>
       </c>
-      <c r="K16" s="3">
+      <c r="N16" s="3">
         <v>100000.0</v>
       </c>
-      <c r="L16" s="3"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O16" s="3"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>15</v>
       </c>
@@ -5997,15 +6148,18 @@
         <v>34.0</v>
       </c>
       <c r="I17" s="3"/>
-      <c r="J17" s="3">
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
+      <c r="M17" s="3">
         <v>100000.0</v>
       </c>
-      <c r="K17" s="3">
+      <c r="N17" s="3">
         <v>100000.0</v>
       </c>
-      <c r="L17" s="3"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O17" s="3"/>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>16</v>
       </c>
@@ -6031,15 +6185,18 @@
         <v>34.0</v>
       </c>
       <c r="I18" s="3"/>
-      <c r="J18" s="3">
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
+      <c r="M18" s="3">
         <v>100000.0</v>
       </c>
-      <c r="K18" s="3">
+      <c r="N18" s="3">
         <v>100000.0</v>
       </c>
-      <c r="L18" s="3"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O18" s="3"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>17</v>
       </c>
@@ -6065,15 +6222,18 @@
         <v>34.0</v>
       </c>
       <c r="I19" s="3"/>
-      <c r="J19" s="3">
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
+      <c r="L19" s="3"/>
+      <c r="M19" s="3">
         <v>100000.0</v>
       </c>
-      <c r="K19" s="3">
+      <c r="N19" s="3">
         <v>100000.0</v>
       </c>
-      <c r="L19" s="3"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O19" s="3"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>18</v>
       </c>
@@ -6099,15 +6259,18 @@
         <v>34.0</v>
       </c>
       <c r="I20" s="3"/>
-      <c r="J20" s="3">
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="3"/>
+      <c r="M20" s="3">
         <v>100000.0</v>
       </c>
-      <c r="K20" s="3">
+      <c r="N20" s="3">
         <v>100000.0</v>
       </c>
-      <c r="L20" s="3"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O20" s="3"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>19</v>
       </c>
@@ -6133,15 +6296,18 @@
         <v>34.0</v>
       </c>
       <c r="I21" s="3"/>
-      <c r="J21" s="3">
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
+      <c r="M21" s="3">
         <v>100000.0</v>
       </c>
-      <c r="K21" s="3">
+      <c r="N21" s="3">
         <v>100000.0</v>
       </c>
-      <c r="L21" s="3"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O21" s="3"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>20</v>
       </c>
@@ -6167,15 +6333,18 @@
         <v>34.0</v>
       </c>
       <c r="I22" s="3"/>
-      <c r="J22" s="3">
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+      <c r="M22" s="3">
         <v>100000.0</v>
       </c>
-      <c r="K22" s="3">
+      <c r="N22" s="3">
         <v>100000.0</v>
       </c>
-      <c r="L22" s="3"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O22" s="3"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>21</v>
       </c>
@@ -6201,15 +6370,18 @@
         <v>34.0</v>
       </c>
       <c r="I23" s="3"/>
-      <c r="J23" s="3">
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+      <c r="M23" s="3">
         <v>100000.0</v>
       </c>
-      <c r="K23" s="3">
+      <c r="N23" s="3">
         <v>100000.0</v>
       </c>
-      <c r="L23" s="3"/>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="O23" s="3"/>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>22</v>
       </c>
@@ -6224,8 +6396,11 @@
       <c r="J24" s="3"/>
       <c r="K24" s="3"/>
       <c r="L24" s="3"/>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M24" s="3"/>
+      <c r="N24" s="3"/>
+      <c r="O24" s="3"/>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>23</v>
       </c>
@@ -6240,8 +6415,11 @@
       <c r="J25" s="3"/>
       <c r="K25" s="3"/>
       <c r="L25" s="3"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M25" s="3"/>
+      <c r="N25" s="3"/>
+      <c r="O25" s="3"/>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" s="3">
         <v>24</v>
       </c>
@@ -6256,8 +6434,11 @@
       <c r="J26" s="3"/>
       <c r="K26" s="3"/>
       <c r="L26" s="3"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M26" s="3"/>
+      <c r="N26" s="3"/>
+      <c r="O26" s="3"/>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" s="3">
         <v>25</v>
       </c>
@@ -6272,8 +6453,11 @@
       <c r="J27" s="3"/>
       <c r="K27" s="3"/>
       <c r="L27" s="3"/>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M27" s="3"/>
+      <c r="N27" s="3"/>
+      <c r="O27" s="3"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28" s="3">
         <v>26</v>
       </c>
@@ -6288,8 +6472,11 @@
       <c r="J28" s="3"/>
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M28" s="3"/>
+      <c r="N28" s="3"/>
+      <c r="O28" s="3"/>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A29" s="3">
         <v>27</v>
       </c>
@@ -6304,8 +6491,11 @@
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
       <c r="L29" s="3"/>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M29" s="3"/>
+      <c r="N29" s="3"/>
+      <c r="O29" s="3"/>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A30" s="3">
         <v>28</v>
       </c>
@@ -6320,8 +6510,11 @@
       <c r="J30" s="3"/>
       <c r="K30" s="3"/>
       <c r="L30" s="3"/>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M30" s="3"/>
+      <c r="N30" s="3"/>
+      <c r="O30" s="3"/>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A31" s="3">
         <v>29</v>
       </c>
@@ -6336,8 +6529,11 @@
       <c r="J31" s="3"/>
       <c r="K31" s="3"/>
       <c r="L31" s="3"/>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M31" s="3"/>
+      <c r="N31" s="3"/>
+      <c r="O31" s="3"/>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A32" s="3">
         <v>30</v>
       </c>
@@ -6352,10 +6548,393 @@
       <c r="J32" s="3"/>
       <c r="K32" s="3"/>
       <c r="L32" s="3"/>
+      <c r="M32" s="3"/>
+      <c r="N32" s="3"/>
+      <c r="O32" s="3"/>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A33" s="3">
+        <v>31</v>
+      </c>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+      <c r="J33" s="3"/>
+      <c r="K33" s="3"/>
+      <c r="L33" s="3"/>
+      <c r="M33" s="3"/>
+      <c r="N33" s="3"/>
+      <c r="O33" s="3"/>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A34" s="3">
+        <v>32</v>
+      </c>
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="3"/>
+      <c r="K34" s="3"/>
+      <c r="L34" s="3"/>
+      <c r="M34" s="3"/>
+      <c r="N34" s="3"/>
+      <c r="O34" s="3"/>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A35" s="3">
+        <v>33</v>
+      </c>
+      <c r="B35" s="3"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
+      <c r="I35" s="3"/>
+      <c r="J35" s="3"/>
+      <c r="K35" s="3"/>
+      <c r="L35" s="3"/>
+      <c r="M35" s="3"/>
+      <c r="N35" s="3"/>
+      <c r="O35" s="3"/>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A36" s="3">
+        <v>34</v>
+      </c>
+      <c r="B36" s="3"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="3"/>
+      <c r="E36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="3"/>
+      <c r="J36" s="3"/>
+      <c r="K36" s="3"/>
+      <c r="L36" s="3"/>
+      <c r="M36" s="3"/>
+      <c r="N36" s="3"/>
+      <c r="O36" s="3"/>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A37" s="3">
+        <v>35</v>
+      </c>
+      <c r="B37" s="3"/>
+      <c r="C37" s="3"/>
+      <c r="D37" s="3"/>
+      <c r="E37" s="3"/>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
+      <c r="H37" s="3"/>
+      <c r="I37" s="3"/>
+      <c r="J37" s="3"/>
+      <c r="K37" s="3"/>
+      <c r="L37" s="3"/>
+      <c r="M37" s="3"/>
+      <c r="N37" s="3"/>
+      <c r="O37" s="3"/>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A38" s="3">
+        <v>36</v>
+      </c>
+      <c r="B38" s="3"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
+      <c r="I38" s="3"/>
+      <c r="J38" s="3"/>
+      <c r="K38" s="3"/>
+      <c r="L38" s="3"/>
+      <c r="M38" s="3"/>
+      <c r="N38" s="3"/>
+      <c r="O38" s="3"/>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A39" s="3">
+        <v>37</v>
+      </c>
+      <c r="B39" s="3"/>
+      <c r="C39" s="3"/>
+      <c r="D39" s="3"/>
+      <c r="E39" s="3"/>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
+      <c r="H39" s="3"/>
+      <c r="I39" s="3"/>
+      <c r="J39" s="3"/>
+      <c r="K39" s="3"/>
+      <c r="L39" s="3"/>
+      <c r="M39" s="3"/>
+      <c r="N39" s="3"/>
+      <c r="O39" s="3"/>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A40" s="3">
+        <v>38</v>
+      </c>
+      <c r="B40" s="3"/>
+      <c r="C40" s="3"/>
+      <c r="D40" s="3"/>
+      <c r="E40" s="3"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
+      <c r="I40" s="3"/>
+      <c r="J40" s="3"/>
+      <c r="K40" s="3"/>
+      <c r="L40" s="3"/>
+      <c r="M40" s="3"/>
+      <c r="N40" s="3"/>
+      <c r="O40" s="3"/>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A41" s="3">
+        <v>39</v>
+      </c>
+      <c r="B41" s="3"/>
+      <c r="C41" s="3"/>
+      <c r="D41" s="3"/>
+      <c r="E41" s="3"/>
+      <c r="F41" s="3"/>
+      <c r="G41" s="3"/>
+      <c r="H41" s="3"/>
+      <c r="I41" s="3"/>
+      <c r="J41" s="3"/>
+      <c r="K41" s="3"/>
+      <c r="L41" s="3"/>
+      <c r="M41" s="3"/>
+      <c r="N41" s="3"/>
+      <c r="O41" s="3"/>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A42" s="3">
+        <v>40</v>
+      </c>
+      <c r="B42" s="3"/>
+      <c r="C42" s="3"/>
+      <c r="D42" s="3"/>
+      <c r="E42" s="3"/>
+      <c r="F42" s="3"/>
+      <c r="G42" s="3"/>
+      <c r="H42" s="3"/>
+      <c r="I42" s="3"/>
+      <c r="J42" s="3"/>
+      <c r="K42" s="3"/>
+      <c r="L42" s="3"/>
+      <c r="M42" s="3"/>
+      <c r="N42" s="3"/>
+      <c r="O42" s="3"/>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A43" s="3">
+        <v>41</v>
+      </c>
+      <c r="B43" s="3"/>
+      <c r="C43" s="3"/>
+      <c r="D43" s="3"/>
+      <c r="E43" s="3"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
+      <c r="H43" s="3"/>
+      <c r="I43" s="3"/>
+      <c r="J43" s="3"/>
+      <c r="K43" s="3"/>
+      <c r="L43" s="3"/>
+      <c r="M43" s="3"/>
+      <c r="N43" s="3"/>
+      <c r="O43" s="3"/>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A44" s="3">
+        <v>42</v>
+      </c>
+      <c r="B44" s="3"/>
+      <c r="C44" s="3"/>
+      <c r="D44" s="3"/>
+      <c r="E44" s="3"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
+      <c r="H44" s="3"/>
+      <c r="I44" s="3"/>
+      <c r="J44" s="3"/>
+      <c r="K44" s="3"/>
+      <c r="L44" s="3"/>
+      <c r="M44" s="3"/>
+      <c r="N44" s="3"/>
+      <c r="O44" s="3"/>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A45" s="3">
+        <v>43</v>
+      </c>
+      <c r="B45" s="3"/>
+      <c r="C45" s="3"/>
+      <c r="D45" s="3"/>
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
+      <c r="I45" s="3"/>
+      <c r="J45" s="3"/>
+      <c r="K45" s="3"/>
+      <c r="L45" s="3"/>
+      <c r="M45" s="3"/>
+      <c r="N45" s="3"/>
+      <c r="O45" s="3"/>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A46" s="3">
+        <v>44</v>
+      </c>
+      <c r="B46" s="3"/>
+      <c r="C46" s="3"/>
+      <c r="D46" s="3"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+      <c r="H46" s="3"/>
+      <c r="I46" s="3"/>
+      <c r="J46" s="3"/>
+      <c r="K46" s="3"/>
+      <c r="L46" s="3"/>
+      <c r="M46" s="3"/>
+      <c r="N46" s="3"/>
+      <c r="O46" s="3"/>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A47" s="3">
+        <v>45</v>
+      </c>
+      <c r="B47" s="3"/>
+      <c r="C47" s="3"/>
+      <c r="D47" s="3"/>
+      <c r="E47" s="3"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
+      <c r="H47" s="3"/>
+      <c r="I47" s="3"/>
+      <c r="J47" s="3"/>
+      <c r="K47" s="3"/>
+      <c r="L47" s="3"/>
+      <c r="M47" s="3"/>
+      <c r="N47" s="3"/>
+      <c r="O47" s="3"/>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A48" s="3">
+        <v>46</v>
+      </c>
+      <c r="B48" s="3"/>
+      <c r="C48" s="3"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+      <c r="I48" s="3"/>
+      <c r="J48" s="3"/>
+      <c r="K48" s="3"/>
+      <c r="L48" s="3"/>
+      <c r="M48" s="3"/>
+      <c r="N48" s="3"/>
+      <c r="O48" s="3"/>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A49" s="3">
+        <v>47</v>
+      </c>
+      <c r="B49" s="3"/>
+      <c r="C49" s="3"/>
+      <c r="D49" s="3"/>
+      <c r="E49" s="3"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
+      <c r="I49" s="3"/>
+      <c r="J49" s="3"/>
+      <c r="K49" s="3"/>
+      <c r="L49" s="3"/>
+      <c r="M49" s="3"/>
+      <c r="N49" s="3"/>
+      <c r="O49" s="3"/>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A50" s="3">
+        <v>48</v>
+      </c>
+      <c r="B50" s="3"/>
+      <c r="C50" s="3"/>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="3"/>
+      <c r="I50" s="3"/>
+      <c r="J50" s="3"/>
+      <c r="K50" s="3"/>
+      <c r="L50" s="3"/>
+      <c r="M50" s="3"/>
+      <c r="N50" s="3"/>
+      <c r="O50" s="3"/>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A51" s="3">
+        <v>49</v>
+      </c>
+      <c r="B51" s="3"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="3"/>
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="3"/>
+      <c r="I51" s="3"/>
+      <c r="J51" s="3"/>
+      <c r="K51" s="3"/>
+      <c r="L51" s="3"/>
+      <c r="M51" s="3"/>
+      <c r="N51" s="3"/>
+      <c r="O51" s="3"/>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A52" s="3">
+        <v>50</v>
+      </c>
+      <c r="B52" s="3"/>
+      <c r="C52" s="3"/>
+      <c r="D52" s="3"/>
+      <c r="E52" s="3"/>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
+      <c r="H52" s="3"/>
+      <c r="I52" s="3"/>
+      <c r="J52" s="3"/>
+      <c r="K52" s="3"/>
+      <c r="L52" s="3"/>
+      <c r="M52" s="3"/>
+      <c r="N52" s="3"/>
+      <c r="O52" s="3"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L3:L32" xr:uid="{D1121F3C-F660-0E46-8AEB-8C1F95C55489}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O3:O52" xr:uid="{D1121F3C-F660-0E46-8AEB-8C1F95C55489}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -11980,20 +12559,6 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="Y6:Z6"/>
     <mergeCell ref="AQ4:AR4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
@@ -12010,6 +12575,20 @@
     <mergeCell ref="AH4:AI4"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="Y6:Z6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -13498,20 +14077,6 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="P7:Q7"/>
-    <mergeCell ref="AB7:AC7"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="S7:T7"/>
-    <mergeCell ref="M7:N7"/>
     <mergeCell ref="S4:T4"/>
     <mergeCell ref="AQ7:AR7"/>
     <mergeCell ref="AN4:AO4"/>
@@ -13528,6 +14093,20 @@
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="V4:W4"/>
     <mergeCell ref="V7:W7"/>
+    <mergeCell ref="AB7:AC7"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P7:Q7"/>
   </mergeCells>
   <conditionalFormatting sqref="B6 A7:B7">
     <cfRule type="expression" dxfId="19" priority="1">

</xml_diff>